<commit_message>
Add Santana de Parnaíba contracts and update database
</commit_message>
<xml_diff>
--- a/dados/enviadas/Educantes.xlsx
+++ b/dados/enviadas/Educantes.xlsx
@@ -18,9 +18,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="[$R$-416] #,##0.00"/>
-    <numFmt numFmtId="165" formatCode="DD/MM/YYYY"/>
+  <numFmts count="3">
+    <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
+    <numFmt numFmtId="165" formatCode="[$R$-416] #,##0.00"/>
+    <numFmt numFmtId="166" formatCode="DD/MM/YYYY"/>
   </numFmts>
   <fonts count="3">
     <font>
@@ -69,21 +70,22 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -456,115 +458,113 @@
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="32" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="23" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="25" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
+    <col width="23" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
     <col width="60" customWidth="1" min="9" max="9"/>
     <col width="59" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>CLIENTE</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>ITEM</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>MODALIDADE</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>VALOR_ESTIMADO</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>ORGAO</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>DATA_DISPUTA</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="H1" s="3" t="inlineStr">
         <is>
           <t>PORTAL</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="I1" s="3" t="inlineStr">
         <is>
           <t>LINK_PORTAL</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="J1" s="3" t="inlineStr">
         <is>
           <t>LINK_PNCP</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
+      <c r="A2" s="4" t="inlineStr">
         <is>
           <t>Educantes</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>122/2026</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>Tradução - Inglês e espanhol</t>
-        </is>
-      </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>Dispensa</t>
-        </is>
-      </c>
-      <c r="E2" s="4" t="n">
-        <v>30600</v>
-      </c>
-      <c r="F2" s="3" t="inlineStr">
-        <is>
-          <t>MINISTERIO DA FAZENDA</t>
-        </is>
-      </c>
-      <c r="G2" s="5" t="inlineStr">
-        <is>
-          <t>19/10/2026</t>
-        </is>
-      </c>
-      <c r="H2" s="3" t="inlineStr">
-        <is>
-          <t>ComprasGov</t>
-        </is>
-      </c>
-      <c r="I2" s="3" t="inlineStr">
-        <is>
-          <t>https://cnetmobile.estaleiro.serpro.gov.br/comprasnet-web/public/compras/acompanhamento-compra?compra=17013306001222026</t>
-        </is>
-      </c>
-      <c r="J2" s="3" t="inlineStr">
-        <is>
-          <t>https://pncp.gov.br/app/editais/00394460000141/2026/691</t>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>172/2026</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>Plataforma de idiomas</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>Pregão - Eletrônico</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="n">
+        <v>850000</v>
+      </c>
+      <c r="F2" s="4" t="inlineStr">
+        <is>
+          <t>MUNICIPIO DE SANTANA DE PARNAIBA</t>
+        </is>
+      </c>
+      <c r="G2" s="6" t="n">
+        <v>46308.39583333334</v>
+      </c>
+      <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>Portal de Compras Públicas</t>
+        </is>
+      </c>
+      <c r="I2" s="4" t="inlineStr">
+        <is>
+          <t>https://www.portaldecompraspublicas.com.br/processos/SP/Prefeitura-Municipal-de-Santana-de-Parnaiba-1139/PE-172-2026-2026-514224</t>
+        </is>
+      </c>
+      <c r="J2" s="4" t="inlineStr">
+        <is>
+          <t>https://pncp.gov.br/app/editais/46522983000127/2026/355</t>
         </is>
       </c>
     </row>

</xml_diff>